<commit_message>
Use official SPXTR returns instead of FMP/SPY for benchmark
The backtest was computing S&P 500 benchmark returns by querying FMP for
SPY ETF data, which systematically understated returns (especially in
strong rally years like 2003, 2009, 2013). Replaced with hardcoded
official S&P 500 Total Return Index (SPXTR) calendar-year returns
cross-referenced from multiple authoritative sources.

This corrects the benchmark from +560% to +653% cumulative (2000-2025),
narrowing portfolio excess return from +117% to +25%.

Also includes: removal of old data-old/ CSVs, updated results files,
turnover analyzer updates, and new return attribution output.
</commit_message>
<xml_diff>
--- a/results-excel/Portfolio_individual_stock_returns.xlsx
+++ b/results-excel/Portfolio_individual_stock_returns.xlsx
@@ -7,32 +7,32 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1999" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2000" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2001" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2002" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="2003" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="2004" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="2005" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="2006" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="2007" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="2008" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="2009" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="2010" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="2011" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="2012" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="2013" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="2014" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="2015" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="2016" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="2017" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="2018" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="2019" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="2020" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="2021" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="2022" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="2023" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="2024" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="2000" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="2001" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2002" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="2003" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2004" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2005" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2006" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2007" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2008" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2009" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2010" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2011" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2012" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2013" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="2014" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="2015" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="2016" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="2017" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="2018" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="2019" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="2020" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="2021" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="2022" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="2023" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="2024" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="2025" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -444,7 +444,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 1999 (Returns: 2000)</t>
+          <t>Portfolio Snapshot — 2000 (S&amp;P 1999 snapshot)</t>
         </is>
       </c>
     </row>
@@ -930,9 +930,15 @@
       <c r="G14" t="n">
         <v>2.157682680286392</v>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>-35.75</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-35.75</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1004,9 +1010,15 @@
       <c r="G16" t="n">
         <v>1.811264425817881</v>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>21.74</v>
+      </c>
+      <c r="I16" t="n">
+        <v>21.74</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1078,9 +1090,15 @@
       <c r="G18" t="n">
         <v>1.435749260495318</v>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>-11.05</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-13.7</v>
+      </c>
+      <c r="J18" t="n">
+        <v>2.6</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1112,9 +1130,15 @@
       <c r="G19" t="n">
         <v>1.112399629286843</v>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>-87.34</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-87.34</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1146,9 +1170,15 @@
       <c r="G20" t="n">
         <v>2.220446049250313e-16</v>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>-81</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-82</v>
+      </c>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1220,9 +1250,15 @@
       <c r="G22" t="n">
         <v>1.146879683533986</v>
       </c>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="I22" t="n">
+        <v>-1.4</v>
+      </c>
+      <c r="J22" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1254,9 +1290,15 @@
       <c r="G23" t="n">
         <v>1.117288821807674</v>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>-6.4</v>
+      </c>
+      <c r="I23" t="n">
+        <v>-9.5</v>
+      </c>
+      <c r="J23" t="n">
+        <v>3.1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1488,9 +1530,15 @@
       <c r="G29" t="n">
         <v>0.9557779097495049</v>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>-69.87</v>
+      </c>
+      <c r="I29" t="n">
+        <v>-69.87</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1642,9 +1690,15 @@
       <c r="G33" t="n">
         <v>2.220446049250313e-16</v>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>-73.5</v>
+      </c>
+      <c r="I33" t="n">
+        <v>-73.5</v>
+      </c>
+      <c r="J33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1756,9 +1810,15 @@
       <c r="G36" t="n">
         <v>2.220446049250313e-16</v>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="H36" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="I36" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J36" t="n">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1830,9 +1890,15 @@
       <c r="G38" t="n">
         <v>2.220446049250313e-16</v>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
+      <c r="H38" t="n">
+        <v>-65.81</v>
+      </c>
+      <c r="I38" t="n">
+        <v>-65.81</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1944,9 +2010,15 @@
       <c r="G41" t="n">
         <v>2.220446049250313e-16</v>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
+      <c r="H41" t="n">
+        <v>-28.01</v>
+      </c>
+      <c r="I41" t="n">
+        <v>-28.01</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -2458,9 +2530,15 @@
       <c r="G54" t="n">
         <v>2.220446049250313e-16</v>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
+      <c r="H54" t="n">
+        <v>36.96</v>
+      </c>
+      <c r="I54" t="n">
+        <v>35</v>
+      </c>
+      <c r="J54" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2732,9 +2810,15 @@
       <c r="G61" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
+      <c r="H61" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="I61" t="n">
+        <v>61.9</v>
+      </c>
+      <c r="J61" t="n">
+        <v>2.3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2766,9 +2850,15 @@
       <c r="G62" t="n">
         <v>0</v>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
+      <c r="H62" t="n">
+        <v>-22.7</v>
+      </c>
+      <c r="I62" t="n">
+        <v>-22.7</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2827,7 +2917,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2008 (Returns: 2009)</t>
+          <t>Portfolio Snapshot — 2009 (S&amp;P 2008 snapshot)</t>
         </is>
       </c>
     </row>
@@ -3593,9 +3683,15 @@
       <c r="G21" t="n">
         <v>1.271247500745847</v>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>31.26</v>
+      </c>
+      <c r="I21" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="J21" t="n">
+        <v>3.1</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3907,9 +4003,15 @@
       <c r="G29" t="n">
         <v>0.9811454657521073</v>
       </c>
-      <c r="H29" t="inlineStr"/>
-      <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr"/>
+      <c r="H29" t="n">
+        <v>17.74</v>
+      </c>
+      <c r="I29" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5288,7 +5390,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2009 (Returns: 2010)</t>
+          <t>Portfolio Snapshot — 2010 (S&amp;P 2009 snapshot)</t>
         </is>
       </c>
     </row>
@@ -6494,9 +6596,15 @@
       <c r="G32" t="n">
         <v>0.8984634050253999</v>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>-13.24</v>
+      </c>
+      <c r="I32" t="n">
+        <v>-14.8</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -7728,9 +7836,15 @@
       <c r="G63" t="n">
         <v>5.551115123125783e-17</v>
       </c>
-      <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr"/>
-      <c r="J63" t="inlineStr"/>
+      <c r="H63" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="I63" t="n">
+        <v>31.08</v>
+      </c>
+      <c r="J63" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7749,7 +7863,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2010 (Returns: 2011)</t>
+          <t>Portfolio Snapshot — 2011 (S&amp;P 2010 snapshot)</t>
         </is>
       </c>
     </row>
@@ -9995,9 +10109,15 @@
       <c r="G58" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
+      <c r="H58" t="n">
+        <v>-5.94</v>
+      </c>
+      <c r="I58" t="n">
+        <v>-5.94</v>
+      </c>
+      <c r="J58" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -10216,7 +10336,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2011 (Returns: 2012)</t>
+          <t>Portfolio Snapshot — 2012 (S&amp;P 2011 snapshot)</t>
         </is>
       </c>
     </row>
@@ -11742,9 +11862,15 @@
       <c r="G40" t="n">
         <v>0.7784420063949045</v>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
+      <c r="H40" t="n">
+        <v>17.46</v>
+      </c>
+      <c r="I40" t="n">
+        <v>17.46</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -12683,7 +12809,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2012 (Returns: 2013)</t>
+          <t>Portfolio Snapshot — 2013 (S&amp;P 2012 snapshot)</t>
         </is>
       </c>
     </row>
@@ -14089,9 +14215,15 @@
       <c r="G37" t="n">
         <v>0.837442972898255</v>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
+      <c r="H37" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="I37" t="n">
+        <v>-0.59</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -14203,9 +14335,15 @@
       <c r="G40" t="n">
         <v>0.8081749221448347</v>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
+      <c r="H40" t="n">
+        <v>57.18</v>
+      </c>
+      <c r="I40" t="n">
+        <v>57.18</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -15144,7 +15282,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2013 (Returns: 2014)</t>
+          <t>Portfolio Snapshot — 2014 (S&amp;P 2013 snapshot)</t>
         </is>
       </c>
     </row>
@@ -16550,9 +16688,15 @@
       <c r="G37" t="n">
         <v>0.8372585725038002</v>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
+      <c r="H37" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="I37" t="n">
+        <v>9.99</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -17611,7 +17755,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2014 (Returns: 2015)</t>
+          <t>Portfolio Snapshot — 2015 (S&amp;P 2014 snapshot)</t>
         </is>
       </c>
     </row>
@@ -20084,7 +20228,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2015 (Returns: 2016)</t>
+          <t>Portfolio Snapshot — 2016 (S&amp;P 2015 snapshot)</t>
         </is>
       </c>
     </row>
@@ -22557,7 +22701,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2016 (Returns: 2017)</t>
+          <t>Portfolio Snapshot — 2017 (S&amp;P 2016 snapshot)</t>
         </is>
       </c>
     </row>
@@ -25030,7 +25174,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2017 (Returns: 2018)</t>
+          <t>Portfolio Snapshot — 2018 (S&amp;P 2017 snapshot)</t>
         </is>
       </c>
     </row>
@@ -27503,7 +27647,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2000 (Returns: 2001)</t>
+          <t>Portfolio Snapshot — 2001 (S&amp;P 2000 snapshot)</t>
         </is>
       </c>
     </row>
@@ -28069,9 +28213,15 @@
       <c r="G16" t="n">
         <v>1.582253343493732</v>
       </c>
-      <c r="H16" t="inlineStr"/>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>-55.87</v>
+      </c>
+      <c r="I16" t="n">
+        <v>-55.87</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -28103,9 +28253,15 @@
       <c r="G17" t="n">
         <v>1.482812003455572</v>
       </c>
-      <c r="H17" t="inlineStr"/>
-      <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>-2</v>
+      </c>
+      <c r="I17" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -28217,9 +28373,15 @@
       <c r="G20" t="n">
         <v>1.378025836281352</v>
       </c>
-      <c r="H20" t="inlineStr"/>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>-5.09</v>
+      </c>
+      <c r="I20" t="n">
+        <v>-8.1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -28651,9 +28813,15 @@
       <c r="G31" t="n">
         <v>1.088658041005976</v>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>-99.27</v>
+      </c>
+      <c r="I31" t="n">
+        <v>-99.27</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -28805,9 +28973,15 @@
       <c r="G35" t="n">
         <v>0.9463900092911879</v>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
+      <c r="H35" t="n">
+        <v>-22.89</v>
+      </c>
+      <c r="I35" t="n">
+        <v>-23.9</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -28999,9 +29173,15 @@
       <c r="G40" t="n">
         <v>0</v>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
+      <c r="H40" t="n">
+        <v>-79.79000000000001</v>
+      </c>
+      <c r="I40" t="n">
+        <v>-79.79000000000001</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -29153,9 +29333,15 @@
       <c r="G44" t="n">
         <v>0.8033177193931345</v>
       </c>
-      <c r="H44" t="inlineStr"/>
-      <c r="I44" t="inlineStr"/>
-      <c r="J44" t="inlineStr"/>
+      <c r="H44" t="n">
+        <v>55.87</v>
+      </c>
+      <c r="I44" t="n">
+        <v>55.87</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -29187,9 +29373,15 @@
       <c r="G45" t="n">
         <v>0.7864887875552324</v>
       </c>
-      <c r="H45" t="inlineStr"/>
-      <c r="I45" t="inlineStr"/>
-      <c r="J45" t="inlineStr"/>
+      <c r="H45" t="n">
+        <v>-53.2</v>
+      </c>
+      <c r="I45" t="n">
+        <v>-53.4</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -29221,9 +29413,15 @@
       <c r="G46" t="n">
         <v>0</v>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
+      <c r="H46" t="n">
+        <v>-17.11</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-20.6</v>
+      </c>
+      <c r="J46" t="n">
+        <v>3.5</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -29335,9 +29533,15 @@
       <c r="G49" t="n">
         <v>0</v>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
+      <c r="H49" t="n">
+        <v>-76.68000000000001</v>
+      </c>
+      <c r="I49" t="n">
+        <v>-76.68000000000001</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -29449,9 +29653,15 @@
       <c r="G52" t="n">
         <v>0</v>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
+      <c r="H52" t="n">
+        <v>-35.92</v>
+      </c>
+      <c r="I52" t="n">
+        <v>-37.4</v>
+      </c>
+      <c r="J52" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -29523,9 +29733,15 @@
       <c r="G54" t="n">
         <v>0</v>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
+      <c r="H54" t="n">
+        <v>-29.32</v>
+      </c>
+      <c r="I54" t="n">
+        <v>-30.3</v>
+      </c>
+      <c r="J54" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -29637,9 +29853,15 @@
       <c r="G57" t="n">
         <v>0</v>
       </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
+      <c r="H57" t="n">
+        <v>-5.85</v>
+      </c>
+      <c r="I57" t="n">
+        <v>-5.85</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -29898,7 +30120,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2018 (Returns: 2019)</t>
+          <t>Portfolio Snapshot — 2019 (S&amp;P 2018 snapshot)</t>
         </is>
       </c>
     </row>
@@ -32371,7 +32593,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2019 (Returns: 2020)</t>
+          <t>Portfolio Snapshot — 2020 (S&amp;P 2019 snapshot)</t>
         </is>
       </c>
     </row>
@@ -34844,7 +35066,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2020 (Returns: 2021)</t>
+          <t>Portfolio Snapshot — 2021 (S&amp;P 2020 snapshot)</t>
         </is>
       </c>
     </row>
@@ -37317,7 +37539,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2021 (Returns: 2022)</t>
+          <t>Portfolio Snapshot — 2022 (S&amp;P 2021 snapshot)</t>
         </is>
       </c>
     </row>
@@ -39790,7 +40012,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2022 (Returns: 2023)</t>
+          <t>Portfolio Snapshot — 2023 (S&amp;P 2022 snapshot)</t>
         </is>
       </c>
     </row>
@@ -42263,7 +42485,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2023 (Returns: 2024)</t>
+          <t>Portfolio Snapshot — 2024 (S&amp;P 2023 snapshot)</t>
         </is>
       </c>
     </row>
@@ -44736,7 +44958,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2024 (Returns: 2025)</t>
+          <t>Portfolio Snapshot — 2025 (S&amp;P 2024 snapshot)</t>
         </is>
       </c>
     </row>
@@ -47209,7 +47431,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2001 (Returns: 2002)</t>
+          <t>Portfolio Snapshot — 2002 (S&amp;P 2001 snapshot)</t>
         </is>
       </c>
     </row>
@@ -47695,9 +47917,15 @@
       <c r="G14" t="n">
         <v>1.994016675203358</v>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>-7.27</v>
+      </c>
+      <c r="I14" t="n">
+        <v>-10.3</v>
+      </c>
+      <c r="J14" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -47889,9 +48117,15 @@
       <c r="G19" t="n">
         <v>1.55036894896427</v>
       </c>
-      <c r="H19" t="inlineStr"/>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>-37.6</v>
+      </c>
+      <c r="I19" t="n">
+        <v>-39.1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -47963,9 +48197,15 @@
       <c r="G21" t="n">
         <v>1.484880315430633</v>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>-7.7</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-7.7</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -48477,9 +48717,15 @@
       <c r="G34" t="n">
         <v>0.8449479794829342</v>
       </c>
-      <c r="H34" t="inlineStr"/>
-      <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr"/>
+      <c r="H34" t="n">
+        <v>-26.04</v>
+      </c>
+      <c r="I34" t="n">
+        <v>-27.4</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1.3</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -48551,9 +48797,15 @@
       <c r="G36" t="n">
         <v>0.8174903132202564</v>
       </c>
-      <c r="H36" t="inlineStr"/>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr"/>
+      <c r="H36" t="n">
+        <v>19.52</v>
+      </c>
+      <c r="I36" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="J36" t="n">
+        <v>3.3</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -48945,9 +49197,15 @@
       <c r="G46" t="n">
         <v>2.220446049250313e-16</v>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
+      <c r="H46" t="n">
+        <v>-30.36</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-33.6</v>
+      </c>
+      <c r="J46" t="n">
+        <v>3.2</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -48979,9 +49237,15 @@
       <c r="G47" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
+      <c r="H47" t="n">
+        <v>-1.62</v>
+      </c>
+      <c r="I47" t="n">
+        <v>-1.62</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -49133,9 +49397,15 @@
       <c r="G51" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
+      <c r="H51" t="n">
+        <v>5.71</v>
+      </c>
+      <c r="I51" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="J51" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -49167,9 +49437,15 @@
       <c r="G52" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H52" t="inlineStr"/>
-      <c r="I52" t="inlineStr"/>
-      <c r="J52" t="inlineStr"/>
+      <c r="H52" t="n">
+        <v>-36.41</v>
+      </c>
+      <c r="I52" t="n">
+        <v>-37.9</v>
+      </c>
+      <c r="J52" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -49281,9 +49557,15 @@
       <c r="G55" t="n">
         <v>1.665334536937735e-16</v>
       </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
+      <c r="H55" t="n">
+        <v>-4.4</v>
+      </c>
+      <c r="I55" t="n">
+        <v>-7.4</v>
+      </c>
+      <c r="J55" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -49355,9 +49637,15 @@
       <c r="G57" t="n">
         <v>5.551115123125783e-17</v>
       </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
+      <c r="H57" t="n">
+        <v>-99.02</v>
+      </c>
+      <c r="I57" t="n">
+        <v>-99.02</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -49429,9 +49717,15 @@
       <c r="G59" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
+      <c r="H59" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="I59" t="n">
+        <v>7.1</v>
+      </c>
+      <c r="J59" t="n">
+        <v>1.6</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -49463,9 +49757,15 @@
       <c r="G60" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H60" t="inlineStr"/>
-      <c r="I60" t="inlineStr"/>
-      <c r="J60" t="inlineStr"/>
+      <c r="H60" t="n">
+        <v>-74.72</v>
+      </c>
+      <c r="I60" t="n">
+        <v>-74.72</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -49537,9 +49837,15 @@
       <c r="G62" t="n">
         <v>1.665334536937735e-16</v>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
+      <c r="H62" t="n">
+        <v>-30.19</v>
+      </c>
+      <c r="I62" t="n">
+        <v>-33.2</v>
+      </c>
+      <c r="J62" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -49598,7 +49904,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2002 (Returns: 2003)</t>
+          <t>Portfolio Snapshot — 2003 (S&amp;P 2002 snapshot)</t>
         </is>
       </c>
     </row>
@@ -50124,9 +50430,15 @@
       <c r="G15" t="n">
         <v>1.712740876553227</v>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>27.08</v>
+      </c>
+      <c r="I15" t="n">
+        <v>27.08</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -50358,9 +50670,15 @@
       <c r="G21" t="n">
         <v>1.225947446088412</v>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="I21" t="n">
+        <v>27.85</v>
+      </c>
+      <c r="J21" t="n">
+        <v>3.4</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -50632,9 +50950,15 @@
       <c r="G28" t="n">
         <v>1.02453069164796</v>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="I28" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1.6</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -50786,9 +51110,15 @@
       <c r="G32" t="n">
         <v>0.7093728393167466</v>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>27.71</v>
+      </c>
+      <c r="I32" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="J32" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -50900,9 +51230,15 @@
       <c r="G35" t="n">
         <v>0.8113473713790107</v>
       </c>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr"/>
+      <c r="H35" t="n">
+        <v>56.75</v>
+      </c>
+      <c r="I35" t="n">
+        <v>55.4</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -50974,9 +51310,15 @@
       <c r="G37" t="n">
         <v>0.8084482439947458</v>
       </c>
-      <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr"/>
-      <c r="J37" t="inlineStr"/>
+      <c r="H37" t="n">
+        <v>25.26</v>
+      </c>
+      <c r="I37" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="J37" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -51008,9 +51350,15 @@
       <c r="G38" t="n">
         <v>0.8052489572874408</v>
       </c>
-      <c r="H38" t="inlineStr"/>
-      <c r="I38" t="inlineStr"/>
-      <c r="J38" t="inlineStr"/>
+      <c r="H38" t="n">
+        <v>-18.71</v>
+      </c>
+      <c r="I38" t="n">
+        <v>-20.2</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -51082,9 +51430,15 @@
       <c r="G40" t="n">
         <v>0.5576169650953707</v>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr"/>
-      <c r="J40" t="inlineStr"/>
+      <c r="H40" t="n">
+        <v>13.16</v>
+      </c>
+      <c r="I40" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="J40" t="n">
+        <v>4.8</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -51316,9 +51670,15 @@
       <c r="G46" t="n">
         <v>2.220446049250313e-16</v>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
+      <c r="H46" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="I46" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -51510,9 +51870,15 @@
       <c r="G51" t="n">
         <v>0.3366292001791064</v>
       </c>
-      <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr"/>
-      <c r="J51" t="inlineStr"/>
+      <c r="H51" t="n">
+        <v>23.55</v>
+      </c>
+      <c r="I51" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="J51" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -51664,9 +52030,15 @@
       <c r="G55" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
+      <c r="H55" t="n">
+        <v>8.15</v>
+      </c>
+      <c r="I55" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="J55" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -51698,9 +52070,15 @@
       <c r="G56" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H56" t="inlineStr"/>
-      <c r="I56" t="inlineStr"/>
-      <c r="J56" t="inlineStr"/>
+      <c r="H56" t="n">
+        <v>9.44</v>
+      </c>
+      <c r="I56" t="n">
+        <v>7</v>
+      </c>
+      <c r="J56" t="n">
+        <v>2.5</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -51999,7 +52377,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2003 (Returns: 2004)</t>
+          <t>Portfolio Snapshot — 2004 (S&amp;P 2003 snapshot)</t>
         </is>
       </c>
     </row>
@@ -52525,9 +52903,15 @@
       <c r="G15" t="n">
         <v>1.696514499443839</v>
       </c>
-      <c r="H15" t="inlineStr"/>
-      <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>24.01</v>
+      </c>
+      <c r="I15" t="n">
+        <v>24.01</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -53159,9 +53543,15 @@
       <c r="G31" t="n">
         <v>1.081109562275921</v>
       </c>
-      <c r="H31" t="inlineStr"/>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr"/>
+      <c r="H31" t="n">
+        <v>3.12</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1.4</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -53233,9 +53623,15 @@
       <c r="G33" t="n">
         <v>0.9938409656396701</v>
       </c>
-      <c r="H33" t="inlineStr"/>
-      <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr"/>
+      <c r="H33" t="n">
+        <v>12.78</v>
+      </c>
+      <c r="I33" t="n">
+        <v>9.800000000000001</v>
+      </c>
+      <c r="J33" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -53867,9 +54263,15 @@
       <c r="G49" t="n">
         <v>-1.110223024625157e-16</v>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
+      <c r="H49" t="n">
+        <v>-18</v>
+      </c>
+      <c r="I49" t="n">
+        <v>-18</v>
+      </c>
+      <c r="J49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -54061,9 +54463,15 @@
       <c r="G54" t="n">
         <v>0</v>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
+      <c r="H54" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="I54" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="J54" t="n">
+        <v>3.6</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -54095,9 +54503,15 @@
       <c r="G55" t="n">
         <v>-1.110223024625157e-16</v>
       </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
+      <c r="H55" t="n">
+        <v>-0.88</v>
+      </c>
+      <c r="I55" t="n">
+        <v>-3.1</v>
+      </c>
+      <c r="J55" t="n">
+        <v>2.2</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -54169,9 +54583,15 @@
       <c r="G57" t="n">
         <v>0</v>
       </c>
-      <c r="H57" t="inlineStr"/>
-      <c r="I57" t="inlineStr"/>
-      <c r="J57" t="inlineStr"/>
+      <c r="H57" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="I57" t="n">
+        <v>-2.4</v>
+      </c>
+      <c r="J57" t="n">
+        <v>4.3</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -54243,9 +54663,15 @@
       <c r="G59" t="n">
         <v>0</v>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
+      <c r="H59" t="n">
+        <v>3.66</v>
+      </c>
+      <c r="I59" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="J59" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -54317,9 +54743,15 @@
       <c r="G61" t="n">
         <v>0</v>
       </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
+      <c r="H61" t="n">
+        <v>-1.95</v>
+      </c>
+      <c r="I61" t="n">
+        <v>-3.5</v>
+      </c>
+      <c r="J61" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -54418,7 +54850,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2004 (Returns: 2005)</t>
+          <t>Portfolio Snapshot — 2005 (S&amp;P 2004 snapshot)</t>
         </is>
       </c>
     </row>
@@ -55464,9 +55896,15 @@
       <c r="G28" t="n">
         <v>1.008984416357769</v>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr"/>
+      <c r="H28" t="n">
+        <v>8.27</v>
+      </c>
+      <c r="I28" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>2.2</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -55618,9 +56056,15 @@
       <c r="G32" t="n">
         <v>0.9198460285746315</v>
       </c>
-      <c r="H32" t="inlineStr"/>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr"/>
+      <c r="H32" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="I32" t="n">
+        <v>2.62</v>
+      </c>
+      <c r="J32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -56052,9 +56496,15 @@
       <c r="G43" t="n">
         <v>0</v>
       </c>
-      <c r="H43" t="inlineStr"/>
-      <c r="I43" t="inlineStr"/>
-      <c r="J43" t="inlineStr"/>
+      <c r="H43" t="n">
+        <v>-28.93</v>
+      </c>
+      <c r="I43" t="n">
+        <v>-28.93</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -56246,9 +56696,15 @@
       <c r="G48" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
+      <c r="H48" t="n">
+        <v>4.29</v>
+      </c>
+      <c r="I48" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="J48" t="n">
+        <v>3.7</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -56640,9 +57096,15 @@
       <c r="G58" t="n">
         <v>2.775557561562891e-16</v>
       </c>
-      <c r="H58" t="inlineStr"/>
-      <c r="I58" t="inlineStr"/>
-      <c r="J58" t="inlineStr"/>
+      <c r="H58" t="n">
+        <v>14.77</v>
+      </c>
+      <c r="I58" t="n">
+        <v>13</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1.8</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -56674,9 +57136,15 @@
       <c r="G59" t="n">
         <v>-1.665334536937735e-16</v>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
+      <c r="H59" t="n">
+        <v>1.77</v>
+      </c>
+      <c r="I59" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="J59" t="n">
+        <v>4.5</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -56788,9 +57256,15 @@
       <c r="G62" t="n">
         <v>5.551115123125783e-17</v>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
+      <c r="H62" t="n">
+        <v>-16.07</v>
+      </c>
+      <c r="I62" t="n">
+        <v>-16.07</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -56849,7 +57323,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2005 (Returns: 2006)</t>
+          <t>Portfolio Snapshot — 2006 (S&amp;P 2005 snapshot)</t>
         </is>
       </c>
     </row>
@@ -57615,9 +58089,15 @@
       <c r="G21" t="n">
         <v>1.288690540891775</v>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>-16.23</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-16.23</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -58409,9 +58889,15 @@
       <c r="G41" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H41" t="inlineStr"/>
-      <c r="I41" t="inlineStr"/>
-      <c r="J41" t="inlineStr"/>
+      <c r="H41" t="n">
+        <v>11.79</v>
+      </c>
+      <c r="I41" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="J41" t="n">
+        <v>4.1</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -58643,9 +59129,15 @@
       <c r="G47" t="n">
         <v>0</v>
       </c>
-      <c r="H47" t="inlineStr"/>
-      <c r="I47" t="inlineStr"/>
-      <c r="J47" t="inlineStr"/>
+      <c r="H47" t="n">
+        <v>-11.45</v>
+      </c>
+      <c r="I47" t="n">
+        <v>-13.5</v>
+      </c>
+      <c r="J47" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -58717,9 +59209,15 @@
       <c r="G49" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
+      <c r="H49" t="n">
+        <v>38.82</v>
+      </c>
+      <c r="I49" t="n">
+        <v>37</v>
+      </c>
+      <c r="J49" t="n">
+        <v>1.8</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -58751,9 +59249,15 @@
       <c r="G50" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H50" t="inlineStr"/>
-      <c r="I50" t="inlineStr"/>
-      <c r="J50" t="inlineStr"/>
+      <c r="H50" t="n">
+        <v>9.51</v>
+      </c>
+      <c r="I50" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="J50" t="n">
+        <v>2.2</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -59185,9 +59689,15 @@
       <c r="G61" t="n">
         <v>0</v>
       </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
+      <c r="H61" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="I61" t="n">
+        <v>75.5</v>
+      </c>
+      <c r="J61" t="n">
+        <v>4.3</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -59219,9 +59729,15 @@
       <c r="G62" t="n">
         <v>1.176836406102666e-14</v>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
+      <c r="H62" t="n">
+        <v>-37.57</v>
+      </c>
+      <c r="I62" t="n">
+        <v>-37.57</v>
+      </c>
+      <c r="J62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -59280,7 +59796,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2006 (Returns: 2007)</t>
+          <t>Portfolio Snapshot — 2007 (S&amp;P 2006 snapshot)</t>
         </is>
       </c>
     </row>
@@ -59926,9 +60442,15 @@
       <c r="G18" t="n">
         <v>1.475732316656571</v>
       </c>
-      <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>-29.91</v>
+      </c>
+      <c r="I18" t="n">
+        <v>-33.22</v>
+      </c>
+      <c r="J18" t="n">
+        <v>4.2</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -61040,9 +61562,15 @@
       <c r="G46" t="n">
         <v>0</v>
       </c>
-      <c r="H46" t="inlineStr"/>
-      <c r="I46" t="inlineStr"/>
-      <c r="J46" t="inlineStr"/>
+      <c r="H46" t="n">
+        <v>-35.1</v>
+      </c>
+      <c r="I46" t="n">
+        <v>-35.1</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -61114,9 +61642,15 @@
       <c r="G48" t="n">
         <v>0</v>
       </c>
-      <c r="H48" t="inlineStr"/>
-      <c r="I48" t="inlineStr"/>
-      <c r="J48" t="inlineStr"/>
+      <c r="H48" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="I48" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="J48" t="n">
+        <v>5.38</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -61148,9 +61682,15 @@
       <c r="G49" t="n">
         <v>0</v>
       </c>
-      <c r="H49" t="inlineStr"/>
-      <c r="I49" t="inlineStr"/>
-      <c r="J49" t="inlineStr"/>
+      <c r="H49" t="n">
+        <v>-41.32</v>
+      </c>
+      <c r="I49" t="n">
+        <v>-43.7</v>
+      </c>
+      <c r="J49" t="n">
+        <v>2.4</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -61382,9 +61922,15 @@
       <c r="G55" t="n">
         <v>0</v>
       </c>
-      <c r="H55" t="inlineStr"/>
-      <c r="I55" t="inlineStr"/>
-      <c r="J55" t="inlineStr"/>
+      <c r="H55" t="n">
+        <v>-14.04</v>
+      </c>
+      <c r="I55" t="n">
+        <v>-16.1</v>
+      </c>
+      <c r="J55" t="n">
+        <v>2.1</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -61616,9 +62162,15 @@
       <c r="G61" t="n">
         <v>0</v>
       </c>
-      <c r="H61" t="inlineStr"/>
-      <c r="I61" t="inlineStr"/>
-      <c r="J61" t="inlineStr"/>
+      <c r="H61" t="n">
+        <v>-2.31</v>
+      </c>
+      <c r="I61" t="n">
+        <v>-2.31</v>
+      </c>
+      <c r="J61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -61650,9 +62202,15 @@
       <c r="G62" t="n">
         <v>3.33066907387547e-16</v>
       </c>
-      <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr"/>
-      <c r="J62" t="inlineStr"/>
+      <c r="H62" t="n">
+        <v>-30.12</v>
+      </c>
+      <c r="I62" t="n">
+        <v>-32.1</v>
+      </c>
+      <c r="J62" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -61711,7 +62269,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Portfolio Snapshot — 2007 (Returns: 2008)</t>
+          <t>Portfolio Snapshot — 2008 (S&amp;P 2007 snapshot)</t>
         </is>
       </c>
     </row>
@@ -62477,9 +63035,15 @@
       <c r="G21" t="n">
         <v>1.169694166786257</v>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>-84.73</v>
+      </c>
+      <c r="I21" t="n">
+        <v>-84.56</v>
+      </c>
+      <c r="J21" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -62671,9 +63235,15 @@
       <c r="G26" t="n">
         <v>0.9512071340769622</v>
       </c>
-      <c r="H26" t="inlineStr"/>
-      <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr"/>
+      <c r="H26" t="n">
+        <v>-36.54</v>
+      </c>
+      <c r="I26" t="n">
+        <v>-37.01</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.5</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -63785,9 +64355,15 @@
       <c r="G54" t="n">
         <v>1.110223024625157e-16</v>
       </c>
-      <c r="H54" t="inlineStr"/>
-      <c r="I54" t="inlineStr"/>
-      <c r="J54" t="inlineStr"/>
+      <c r="H54" t="n">
+        <v>-14.54</v>
+      </c>
+      <c r="I54" t="n">
+        <v>-17.2</v>
+      </c>
+      <c r="J54" t="n">
+        <v>2.6</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -63979,9 +64555,15 @@
       <c r="G59" t="n">
         <v>3.885780586188048e-16</v>
       </c>
-      <c r="H59" t="inlineStr"/>
-      <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
+      <c r="H59" t="n">
+        <v>-58.22</v>
+      </c>
+      <c r="I59" t="n">
+        <v>-58.22</v>
+      </c>
+      <c r="J59" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">

</xml_diff>